<commit_message>
Optimized for v3.1.3 and v3.1.4
</commit_message>
<xml_diff>
--- a/assets/data/DLT历史数据_适配模型版.xlsx
+++ b/assets/data/DLT历史数据_适配模型版.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2885"/>
+  <dimension ref="A1:H2887"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -75454,6 +75454,58 @@
         <v>5</v>
       </c>
     </row>
+    <row r="2886">
+      <c r="A2886" t="n">
+        <v>26067</v>
+      </c>
+      <c r="B2886" t="n">
+        <v>6</v>
+      </c>
+      <c r="C2886" t="n">
+        <v>16</v>
+      </c>
+      <c r="D2886" t="n">
+        <v>18</v>
+      </c>
+      <c r="E2886" t="n">
+        <v>19</v>
+      </c>
+      <c r="F2886" t="n">
+        <v>28</v>
+      </c>
+      <c r="G2886" t="n">
+        <v>7</v>
+      </c>
+      <c r="H2886" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2887">
+      <c r="A2887" t="n">
+        <v>26068</v>
+      </c>
+      <c r="B2887" t="n">
+        <v>3</v>
+      </c>
+      <c r="C2887" t="n">
+        <v>11</v>
+      </c>
+      <c r="D2887" t="n">
+        <v>12</v>
+      </c>
+      <c r="E2887" t="n">
+        <v>21</v>
+      </c>
+      <c r="F2887" t="n">
+        <v>22</v>
+      </c>
+      <c r="G2887" t="n">
+        <v>6</v>
+      </c>
+      <c r="H2887" t="n">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
 </worksheet>

</xml_diff>